<commit_message>
Completa la referencia de Salazar-Jiménez et al. (2026) y da el título original de los estudios en español
Los coautores salen de la primera página del artículo. Los seis estudios
citados que están escritos en español llevan el título original y la
traducción al inglés entre corchetes, como pide APA 7. Se regeneran el libro
de Excel y el Word.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W48ggkE3iqcgcPHVfB8T9P
</commit_message>
<xml_diff>
--- a/revision-adc/figuras-y-tablas.xlsx
+++ b/revision-adc/figuras-y-tablas.xlsx
@@ -83,7 +83,7 @@
     <t xml:space="preserve">Authors</t>
   </si>
   <si>
-    <t xml:space="preserve">Full author lists come from Crossref, checked against ORCID and the journal page where Crossref was wrong or empty. Five studies still show only the first author and the number of co-authors.</t>
+    <t xml:space="preserve">Full author lists come from Crossref, checked against ORCID and the journal page where Crossref was wrong or empty. Four studies that are not cited in the article still show only the first author and the number of co-authors.</t>
   </si>
   <si>
     <t xml:space="preserve">Figure 1. Two-pass selection of studies</t>
@@ -2855,7 +2855,7 @@
     <t xml:space="preserve">2-s2.0-105044055600</t>
   </si>
   <si>
-    <t xml:space="preserve">Salazar-Jiménez, R., [+2 co-authors]</t>
+    <t xml:space="preserve">Salazar-Jiménez, R., Orellana Fonseca, C., &amp; Fuentes Rodríguez, C.</t>
   </si>
   <si>
     <t xml:space="preserve">INITIAL TEACHER EDUCATION AND DIGITAL CITIZENSHIP: TENSIONS AND CHALLENGES IN SOCIAL STUDIES EDUCATION</t>
@@ -6669,8 +6669,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="96366015"/>
-        <c:axId val="9833932"/>
+        <c:axId val="16762946"/>
+        <c:axId val="70648445"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -6819,11 +6819,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="96366015"/>
-        <c:axId val="9833932"/>
+        <c:axId val="16762946"/>
+        <c:axId val="70648445"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="96366015"/>
+        <c:axId val="16762946"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6889,7 +6889,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9833932"/>
+        <c:crossAx val="70648445"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6897,7 +6897,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9833932"/>
+        <c:axId val="70648445"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6973,7 +6973,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96366015"/>
+        <c:crossAx val="16762946"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7210,11 +7210,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="73393925"/>
-        <c:axId val="74300484"/>
+        <c:axId val="69357757"/>
+        <c:axId val="847900"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="73393925"/>
+        <c:axId val="69357757"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7246,7 +7246,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74300484"/>
+        <c:crossAx val="847900"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7254,7 +7254,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="74300484"/>
+        <c:axId val="847900"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7330,7 +7330,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73393925"/>
+        <c:crossAx val="69357757"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7507,11 +7507,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="60400660"/>
-        <c:axId val="44262111"/>
+        <c:axId val="61354239"/>
+        <c:axId val="30274768"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60400660"/>
+        <c:axId val="61354239"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7543,7 +7543,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44262111"/>
+        <c:crossAx val="30274768"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7551,7 +7551,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44262111"/>
+        <c:axId val="30274768"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7593,7 +7593,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60400660"/>
+        <c:crossAx val="61354239"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8057,11 +8057,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="72911032"/>
-        <c:axId val="7117742"/>
+        <c:axId val="24221863"/>
+        <c:axId val="71366006"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="72911032"/>
+        <c:axId val="24221863"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8093,7 +8093,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7117742"/>
+        <c:crossAx val="71366006"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8101,7 +8101,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7117742"/>
+        <c:axId val="71366006"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8177,7 +8177,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72911032"/>
+        <c:crossAx val="24221863"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Versión lista para enviar: descripciones cotejadas, página de título completa
- Cotejo de las descripciones de los 61 estudios citados con su texto completo
  o su resumen; corrige cuatro descripciones y retira Lo et al. (2024) de la
  tabla 6 (también en el libro de Excel).
- Página de título con afiliación, correo, financiación y enlace a los datos.
- Word del manuscrito, página de título, carta y S4 regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W48ggkE3iqcgcPHVfB8T9P
</commit_message>
<xml_diff>
--- a/revision-adc/figuras-y-tablas.xlsx
+++ b/revision-adc/figuras-y-tablas.xlsx
@@ -672,7 +672,7 @@
     <t xml:space="preserve">Read memes, videos, teaching materials or AI outputs for representation, bias and ideology</t>
   </si>
   <si>
-    <t xml:space="preserve">Elmore &amp; Coleman (2019); Ho &amp; Hafner (2025); Van Poucke (2024); Weninger &amp; Xu (2026)</t>
+    <t xml:space="preserve">Political memes in middle school (Elmore &amp; Coleman, 2019); diversity in airline safety videos (Ho &amp; Hafner, 2025); ideological bias in chatbot answers (Van Poucke, 2024); visual bias in AI images (Weninger &amp; Xu, 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Media production and multimodal composing</t>
@@ -681,7 +681,7 @@
     <t xml:space="preserve">Produce video, stories, posters or multimodal texts that answer dominant narratives</t>
   </si>
   <si>
-    <t xml:space="preserve">Watt (2019); Noble &amp; Gachago (2022); de los Ríos (2018); Damaskinidis et al. (2026)</t>
+    <t xml:space="preserve">Video production in elementary teacher education (Watt, 2019); digital storytelling on District Six (Noble &amp; Gachago, 2022); bilingual Vine making (de los Ríos, 2018); translating a poster campaign on cyberbullying (Damaskinidis et al., 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Virtual exchange</t>
@@ -690,7 +690,7 @@
     <t xml:space="preserve">Work with peers in other countries and examine how platforms shape the exchange</t>
   </si>
   <si>
-    <t xml:space="preserve">Hauck (2019); Bilki et al. (2023); Satar et al. (2023); Ketzer-Nöltge &amp; Markovic (2022)</t>
+    <t xml:space="preserve">Hauck (2019); ELT teacher education (Bilki et al., 2023); multimodal representation (Satar et al., 2023); a COIL project with pre-service teachers (Ketzer-Nöltge &amp; Markovic, 2022)</t>
   </si>
   <si>
     <t xml:space="preserve">Designed modules and inquiry</t>
@@ -699,7 +699,7 @@
     <t xml:space="preserve">Follow a sequence built around a game, a controversy or a writing task</t>
   </si>
   <si>
-    <t xml:space="preserve">Jiménez Torras et al. (2026); Gerlach et al. (2025); Spracklin &amp; Espina (2025); Lo et al. (2024)</t>
+    <t xml:space="preserve">Co-designing a module with indie video games (Jiménez Torras et al., 2026); conspiracy theories in English classes (Gerlach et al., 2025); reflection notebooks on misinformation (Spracklin &amp; Espina, 2025); rating classroom tools for privacy with future primary teachers (Castañeda &amp; Villar-Onrubia, 2023)</t>
   </si>
   <si>
     <t xml:space="preserve">Civic action</t>
@@ -708,7 +708,7 @@
     <t xml:space="preserve">Use digital tools to investigate and act on local or political issues</t>
   </si>
   <si>
-    <t xml:space="preserve">Kwon &amp; de los Ríos (2019); Abowitz &amp; Mamlok (2020); Fernández (2026); Tanksley (2024)</t>
+    <t xml:space="preserve">Civic interrogation in a ninth-grade ethnic studies course (Kwon &amp; de los Ríos, 2019); student activism after the Parkland shooting (Abowitz &amp; Mamlok, 2020); university digital activism in Peru (Fernández, 2026); Black students resisting AI-mediated racism (Tanksley, 2024)</t>
   </si>
   <si>
     <t xml:space="preserve">Table 7. The ten most cited studies</t>
@@ -6703,8 +6703,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="78357086"/>
-        <c:axId val="1060801"/>
+        <c:axId val="26301396"/>
+        <c:axId val="35297810"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -6853,11 +6853,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="78357086"/>
-        <c:axId val="1060801"/>
+        <c:axId val="26301396"/>
+        <c:axId val="35297810"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="78357086"/>
+        <c:axId val="26301396"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6923,7 +6923,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1060801"/>
+        <c:crossAx val="35297810"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6931,7 +6931,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1060801"/>
+        <c:axId val="35297810"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7007,7 +7007,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78357086"/>
+        <c:crossAx val="26301396"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7244,11 +7244,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="2793568"/>
-        <c:axId val="48618844"/>
+        <c:axId val="6108322"/>
+        <c:axId val="96194551"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2793568"/>
+        <c:axId val="6108322"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7280,7 +7280,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="48618844"/>
+        <c:crossAx val="96194551"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7288,7 +7288,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="48618844"/>
+        <c:axId val="96194551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7364,7 +7364,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2793568"/>
+        <c:crossAx val="6108322"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7541,11 +7541,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="19744410"/>
-        <c:axId val="78917623"/>
+        <c:axId val="90360193"/>
+        <c:axId val="18907854"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19744410"/>
+        <c:axId val="90360193"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -7577,7 +7577,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78917623"/>
+        <c:crossAx val="18907854"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7585,7 +7585,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78917623"/>
+        <c:axId val="18907854"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7627,7 +7627,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19744410"/>
+        <c:crossAx val="90360193"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8091,11 +8091,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="60956358"/>
-        <c:axId val="90372988"/>
+        <c:axId val="73224649"/>
+        <c:axId val="66991258"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="60956358"/>
+        <c:axId val="73224649"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8127,7 +8127,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90372988"/>
+        <c:crossAx val="66991258"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8135,7 +8135,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="90372988"/>
+        <c:axId val="66991258"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8211,7 +8211,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60956358"/>
+        <c:crossAx val="73224649"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9523,7 +9523,8 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="90"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9542,7 +9543,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
         <v>208</v>
       </c>
@@ -9553,7 +9554,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
         <v>211</v>
       </c>
@@ -9575,7 +9576,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
         <v>217</v>
       </c>
@@ -9586,7 +9587,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
         <v>220</v>
       </c>

</xml_diff>